<commit_message>
Updated Analog Reader to V1.1
Added analog filtering (4.7kOhms res + 1uF cap) on all inputs
</commit_message>
<xml_diff>
--- a/Electronics/PCBs/Analog Reader/BOM.xlsx
+++ b/Electronics/PCBs/Analog Reader/BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
   <si>
     <t>No.</t>
   </si>
@@ -70,6 +70,27 @@
     <t>2</t>
   </si>
   <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>C1,C2,C3,C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16</t>
+  </si>
+  <si>
+    <t>C0603</t>
+  </si>
+  <si>
+    <t>CL10A105KB8NNNC</t>
+  </si>
+  <si>
+    <t>SAMSUNG(三星)</t>
+  </si>
+  <si>
+    <t>C15849</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
     <t>100nF</t>
   </si>
   <si>
@@ -88,7 +109,7 @@
     <t>C49678</t>
   </si>
   <si>
-    <t>3</t>
+    <t>4</t>
   </si>
   <si>
     <t>B4B-PH-K-S(LF)(SN)</t>
@@ -106,10 +127,10 @@
     <t>C131334</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>B7B-PH-K-S(LF)(SN)</t>
+    <t>5</t>
+  </si>
+  <si>
+    <t>B7B-PH</t>
   </si>
   <si>
     <t>CN-SIGNAL</t>
@@ -119,6 +140,27 @@
   </si>
   <si>
     <t>C157981</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>4.7kΩ</t>
+  </si>
+  <si>
+    <t>R1,R2,R3,R4,R5,R6,R7,R8,R9,R10,R11,R12,R13,R14,R15,R16</t>
+  </si>
+  <si>
+    <t>R0603</t>
+  </si>
+  <si>
+    <t>0603WAF4701T5E</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(厚声)</t>
+  </si>
+  <si>
+    <t>C23162</t>
   </si>
 </sst>
 </file>
@@ -495,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -570,7 +612,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -602,7 +644,7 @@
         <v>25</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>
@@ -614,16 +656,16 @@
         <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>17</v>
@@ -631,38 +673,102 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H5" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>